<commit_message>
feat(config)!: migrate modifier configuration to UE operations
Update the schema, generated types, workbook validation, compiler mappings, examples, and runtime tests for the six UE modifier operations.

BREAKING CHANGE: Adopt UE operation names and numeric values. Convert old PercentAdd magnitudes to multipliers and re-export existing configuration packages.
</commit_message>
<xml_diff>
--- a/config/tables/gas.modifier.xlsx
+++ b/config/tables/gas.modifier.xlsx
@@ -1253,7 +1253,7 @@
         <x:v>Mana</x:v>
       </x:c>
       <x:c r="D5" s="5" t="str">
-        <x:v>Add</x:v>
+        <x:v>AddBase</x:v>
       </x:c>
       <x:c r="E5" s="5" t="str">
         <x:v>Flat</x:v>
@@ -1274,7 +1274,7 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="D6" s="5" t="str">
-        <x:v>Add</x:v>
+        <x:v>AddBase</x:v>
       </x:c>
       <x:c r="E6" s="5" t="str">
         <x:v>LinearLevel</x:v>
@@ -1289,7 +1289,7 @@
   </x:sheetData>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="D5:D6">
-      <x:formula1>"Add,PercentAdd,Multiply,Override"</x:formula1>
+      <x:formula1>"AddBase,MultiplyAdditive,DivideAdditive,Override,MultiplyCompound,AddFinal"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="E5:E6">
       <x:formula1>"Flat,LinearLevel"</x:formula1>

</xml_diff>